<commit_message>
added pin usage info
</commit_message>
<xml_diff>
--- a/All-IOPins.xlsx
+++ b/All-IOPins.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sawtelles\Documents\GitHub\Teensy-Odd-and-Ends\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BF21DE72-E386-4CCE-B694-28AF3D079C50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80172C5D-296E-42DC-8FB1-902F17EB3840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="18240" windowHeight="28320" xr2:uid="{207FC95A-C154-4EA4-B2D9-D2F6000D8F44}"/>
   </bookViews>
@@ -969,7 +969,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -989,9 +989,12 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1374,20 +1377,20 @@
       <c r="J2" s="13"/>
       <c r="K2" s="13"/>
     </row>
-    <row r="3" spans="1:11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
         <v>276</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="15"/>
     </row>
     <row r="4" spans="1:11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">

</xml_diff>

<commit_message>
Correct a few pin assignments
</commit_message>
<xml_diff>
--- a/All-IOPins.xlsx
+++ b/All-IOPins.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sawtelles\Documents\GitHub\Teensy-Odd-and-Ends\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71831CA7-D14D-44F9-9788-4C7B3732D427}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{990A2674-8C32-4AA6-9395-73354780FB95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="18240" windowHeight="28320" xr2:uid="{207FC95A-C154-4EA4-B2D9-D2F6000D8F44}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="284">
   <si>
     <t>BIT</t>
   </si>
@@ -879,6 +879,15 @@
   </si>
   <si>
     <t>TX1/MISO1</t>
+  </si>
+  <si>
+    <t>ETH_RST</t>
+  </si>
+  <si>
+    <t>ETH_INT</t>
+  </si>
+  <si>
+    <t>6</t>
   </si>
 </sst>
 </file>
@@ -916,7 +925,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -964,11 +973,73 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -996,6 +1067,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1331,26 +1412,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9656BE50-9C77-4DF8-ABEC-98B97523EA1E}">
   <dimension ref="A1:O47"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.28515625" customWidth="1"/>
-    <col min="2" max="2" width="8.85546875" customWidth="1"/>
-    <col min="3" max="4" width="15.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.28515625" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" customWidth="1"/>
-    <col min="8" max="8" width="6.85546875" customWidth="1"/>
-    <col min="9" max="9" width="9.28515625" customWidth="1"/>
-    <col min="10" max="10" width="15.28515625" customWidth="1"/>
-    <col min="11" max="11" width="12.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="6.85546875" customWidth="1"/>
-    <col min="13" max="13" width="10.7109375" customWidth="1"/>
-    <col min="14" max="14" width="13.85546875" customWidth="1"/>
+    <col min="1" max="1" width="6.33203125" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" customWidth="1"/>
+    <col min="3" max="4" width="15.44140625" customWidth="1"/>
+    <col min="5" max="5" width="10.33203125" customWidth="1"/>
+    <col min="6" max="6" width="16.88671875" customWidth="1"/>
+    <col min="7" max="7" width="13.5546875" customWidth="1"/>
+    <col min="8" max="8" width="6.88671875" customWidth="1"/>
+    <col min="9" max="9" width="9.33203125" customWidth="1"/>
+    <col min="10" max="10" width="15.33203125" customWidth="1"/>
+    <col min="11" max="11" width="12.6640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="6.88671875" customWidth="1"/>
+    <col min="13" max="13" width="10.6640625" customWidth="1"/>
+    <col min="14" max="14" width="13.88671875" customWidth="1"/>
     <col min="15" max="15" width="13" style="1" customWidth="1"/>
-    <col min="16" max="16384" width="9.140625" style="1"/>
+    <col min="16" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>205</v>
       </c>
@@ -1369,7 +1450,7 @@
       <c r="N1" s="12"/>
       <c r="O1" s="8"/>
     </row>
-    <row r="2" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="13" t="s">
         <v>251</v>
       </c>
@@ -1388,7 +1469,7 @@
       <c r="N2" s="14"/>
       <c r="O2" s="9"/>
     </row>
-    <row r="3" spans="1:15" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
         <v>252</v>
       </c>
@@ -1407,7 +1488,7 @@
       <c r="N3" s="16"/>
       <c r="O3" s="9"/>
     </row>
-    <row r="4" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
@@ -1420,7 +1501,7 @@
       <c r="D4" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="17" t="s">
         <v>209</v>
       </c>
       <c r="F4" s="3" t="s">
@@ -1429,7 +1510,7 @@
       <c r="G4" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="H4" s="20" t="s">
         <v>0</v>
       </c>
       <c r="I4" s="4" t="s">
@@ -1454,7 +1535,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="5" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>0</v>
       </c>
@@ -1467,14 +1548,14 @@
       <c r="D5" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="18" t="s">
         <v>95</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>198</v>
       </c>
       <c r="G5" s="1"/>
-      <c r="H5">
+      <c r="H5" s="21">
         <v>0</v>
       </c>
       <c r="I5" s="1" t="s">
@@ -1494,7 +1575,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="6" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <f>A5+1</f>
         <v>1</v>
@@ -1508,14 +1589,14 @@
       <c r="D6" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="18" t="s">
         <v>133</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>246</v>
       </c>
       <c r="G6" s="1"/>
-      <c r="H6">
+      <c r="H6" s="21">
         <f>H5+1</f>
         <v>1</v>
       </c>
@@ -1537,7 +1618,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="7" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <f t="shared" ref="A7:A47" si="0">A6+1</f>
         <v>2</v>
@@ -1551,7 +1632,7 @@
       <c r="D7" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="18" t="s">
         <v>4</v>
       </c>
       <c r="F7" s="2" t="s">
@@ -1560,7 +1641,7 @@
       <c r="G7" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="21">
         <f t="shared" ref="H7:H47" si="1">H6+1</f>
         <v>2</v>
       </c>
@@ -1582,7 +1663,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="8" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -1596,7 +1677,7 @@
       <c r="D8" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="18" t="s">
         <v>2</v>
       </c>
       <c r="F8" s="2" t="s">
@@ -1605,7 +1686,7 @@
       <c r="G8" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="21">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
@@ -1627,7 +1708,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="9" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1639,14 +1720,14 @@
         <v>248</v>
       </c>
       <c r="D9" s="1"/>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="18" t="s">
         <v>134</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>173</v>
       </c>
       <c r="G9" s="1"/>
-      <c r="H9">
+      <c r="H9" s="21">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
@@ -1668,7 +1749,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="10" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1680,14 +1761,14 @@
         <v>249</v>
       </c>
       <c r="D10" s="1"/>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="18" t="s">
         <v>135</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>172</v>
       </c>
       <c r="G10" s="1"/>
-      <c r="H10">
+      <c r="H10" s="21">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
@@ -1709,7 +1790,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="11" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1721,14 +1802,14 @@
         <v>250</v>
       </c>
       <c r="D11" s="1"/>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="18" t="s">
         <v>136</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>174</v>
       </c>
       <c r="G11" s="1"/>
-      <c r="H11">
+      <c r="H11" s="21">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
@@ -1748,7 +1829,7 @@
       </c>
       <c r="N11" s="1"/>
     </row>
-    <row r="12" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1756,18 +1837,15 @@
       <c r="B12" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="C12" s="2">
-        <v>6</v>
-      </c>
       <c r="D12" s="1"/>
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="18" t="s">
         <v>137</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>175</v>
       </c>
       <c r="G12" s="1"/>
-      <c r="H12">
+      <c r="H12" s="21">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
@@ -1787,7 +1865,7 @@
       </c>
       <c r="N12" s="1"/>
     </row>
-    <row r="13" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1795,18 +1873,15 @@
       <c r="B13" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>208</v>
-      </c>
       <c r="D13" s="1"/>
-      <c r="E13" s="1" t="s">
+      <c r="E13" s="18" t="s">
         <v>138</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>176</v>
       </c>
       <c r="G13" s="1"/>
-      <c r="H13">
+      <c r="H13" s="21">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
@@ -1826,7 +1901,7 @@
       </c>
       <c r="N13" s="1"/>
     </row>
-    <row r="14" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1838,14 +1913,14 @@
         <v>94</v>
       </c>
       <c r="D14" s="1"/>
-      <c r="E14" s="1" t="s">
+      <c r="E14" s="18" t="s">
         <v>139</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>177</v>
       </c>
       <c r="G14" s="1"/>
-      <c r="H14">
+      <c r="H14" s="21">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
@@ -1865,7 +1940,7 @@
       </c>
       <c r="N14" s="1"/>
     </row>
-    <row r="15" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1874,17 +1949,17 @@
         <v>12</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>206</v>
+        <v>283</v>
       </c>
       <c r="D15" s="1"/>
-      <c r="E15" s="1" t="s">
+      <c r="E15" s="18" t="s">
         <v>140</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>178</v>
       </c>
       <c r="G15" s="1"/>
-      <c r="H15">
+      <c r="H15" s="21">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
@@ -1904,7 +1979,7 @@
       </c>
       <c r="N15" s="1"/>
     </row>
-    <row r="16" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1912,16 +1987,18 @@
       <c r="B16" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="2"/>
+      <c r="C16" s="2" t="s">
+        <v>208</v>
+      </c>
       <c r="D16" s="1"/>
-      <c r="E16" s="1" t="s">
+      <c r="E16" s="18" t="s">
         <v>141</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>180</v>
       </c>
       <c r="G16" s="1"/>
-      <c r="H16">
+      <c r="H16" s="21">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
@@ -1941,7 +2018,7 @@
       </c>
       <c r="N16" s="1"/>
     </row>
-    <row r="17" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1953,7 +2030,7 @@
         <v>60</v>
       </c>
       <c r="D17" s="1"/>
-      <c r="E17" s="1" t="s">
+      <c r="E17" s="18" t="s">
         <v>45</v>
       </c>
       <c r="F17" s="2" t="s">
@@ -1962,7 +2039,7 @@
       <c r="G17" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="H17">
+      <c r="H17" s="21">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
@@ -1982,7 +2059,7 @@
       </c>
       <c r="N17" s="1"/>
     </row>
-    <row r="18" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1990,9 +2067,11 @@
       <c r="B18" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="C18" s="2"/>
+      <c r="C18" s="2" t="s">
+        <v>206</v>
+      </c>
       <c r="D18" s="1"/>
-      <c r="E18" s="1" t="s">
+      <c r="E18" s="18" t="s">
         <v>47</v>
       </c>
       <c r="F18" s="2" t="s">
@@ -2001,7 +2080,7 @@
       <c r="G18" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="21">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
@@ -2021,7 +2100,7 @@
       </c>
       <c r="N18" s="1"/>
     </row>
-    <row r="19" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2030,15 +2109,17 @@
         <v>148</v>
       </c>
       <c r="C19" s="2"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1" t="s">
+      <c r="D19" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="E19" s="18" t="s">
         <v>142</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>245</v>
       </c>
       <c r="G19" s="1"/>
-      <c r="H19">
+      <c r="H19" s="21">
         <f t="shared" si="1"/>
         <v>14</v>
       </c>
@@ -2058,7 +2139,7 @@
       </c>
       <c r="N19" s="1"/>
     </row>
-    <row r="20" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -2067,15 +2148,17 @@
         <v>149</v>
       </c>
       <c r="C20" s="5"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6" t="s">
+      <c r="D20" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="E20" s="19" t="s">
         <v>143</v>
       </c>
       <c r="F20" s="5" t="s">
         <v>228</v>
       </c>
       <c r="G20" s="6"/>
-      <c r="H20" s="8">
+      <c r="H20" s="22">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
@@ -2096,7 +2179,7 @@
       <c r="N20" s="6"/>
       <c r="O20" s="8"/>
     </row>
-    <row r="21" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -2110,7 +2193,7 @@
       <c r="D21" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="E21" s="18" t="s">
         <v>35</v>
       </c>
       <c r="F21" s="2" t="s">
@@ -2119,7 +2202,7 @@
       <c r="G21" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="H21">
+      <c r="H21" s="21">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
@@ -2141,7 +2224,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="22" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -2155,7 +2238,7 @@
       <c r="D22" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="E22" s="18" t="s">
         <v>33</v>
       </c>
       <c r="F22" s="2" t="s">
@@ -2164,7 +2247,7 @@
       <c r="G22" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="H22">
+      <c r="H22" s="21">
         <f t="shared" si="1"/>
         <v>17</v>
       </c>
@@ -2186,7 +2269,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="23" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -2200,7 +2283,7 @@
       <c r="D23" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="E23" s="18" t="s">
         <v>25</v>
       </c>
       <c r="F23" s="2" t="s">
@@ -2209,7 +2292,7 @@
       <c r="G23" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="H23">
+      <c r="H23" s="21">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
@@ -2231,7 +2314,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="24" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -2245,7 +2328,7 @@
       <c r="D24" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="E24" s="18" t="s">
         <v>27</v>
       </c>
       <c r="F24" s="2" t="s">
@@ -2254,7 +2337,7 @@
       <c r="G24" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="H24">
+      <c r="H24" s="21">
         <f t="shared" si="1"/>
         <v>19</v>
       </c>
@@ -2276,7 +2359,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="25" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -2288,14 +2371,14 @@
         <v>104</v>
       </c>
       <c r="D25" s="1"/>
-      <c r="E25" s="1" t="s">
+      <c r="E25" s="18" t="s">
         <v>77</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>76</v>
       </c>
       <c r="G25" s="1"/>
-      <c r="H25">
+      <c r="H25" s="21">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
@@ -2317,7 +2400,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="26" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -2329,14 +2412,14 @@
         <v>104</v>
       </c>
       <c r="D26" s="1"/>
-      <c r="E26" s="1" t="s">
+      <c r="E26" s="18" t="s">
         <v>79</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>78</v>
       </c>
       <c r="G26" s="1"/>
-      <c r="H26">
+      <c r="H26" s="21">
         <f t="shared" si="1"/>
         <v>21</v>
       </c>
@@ -2358,7 +2441,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="27" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -2370,7 +2453,7 @@
         <v>104</v>
       </c>
       <c r="D27" s="1"/>
-      <c r="E27" s="1" t="s">
+      <c r="E27" s="18" t="s">
         <v>31</v>
       </c>
       <c r="F27" s="2" t="s">
@@ -2379,7 +2462,7 @@
       <c r="G27" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="H27">
+      <c r="H27" s="21">
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
@@ -2401,7 +2484,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="28" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -2413,7 +2496,7 @@
         <v>104</v>
       </c>
       <c r="D28" s="1"/>
-      <c r="E28" s="1" t="s">
+      <c r="E28" s="18" t="s">
         <v>29</v>
       </c>
       <c r="F28" s="2" t="s">
@@ -2422,7 +2505,7 @@
       <c r="G28" s="1" t="s">
         <v>272</v>
       </c>
-      <c r="H28">
+      <c r="H28" s="21">
         <f t="shared" si="1"/>
         <v>23</v>
       </c>
@@ -2444,7 +2527,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="29" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -2456,14 +2539,14 @@
         <v>104</v>
       </c>
       <c r="D29" s="1"/>
-      <c r="E29" s="1" t="s">
+      <c r="E29" s="18" t="s">
         <v>41</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>40</v>
       </c>
       <c r="G29" s="1"/>
-      <c r="H29">
+      <c r="H29" s="21">
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
@@ -2485,7 +2568,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="30" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <f t="shared" si="0"/>
         <v>25</v>
@@ -2497,14 +2580,14 @@
         <v>104</v>
       </c>
       <c r="D30" s="1"/>
-      <c r="E30" s="1" t="s">
+      <c r="E30" s="18" t="s">
         <v>43</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>42</v>
       </c>
       <c r="G30" s="1"/>
-      <c r="H30">
+      <c r="H30" s="21">
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
@@ -2526,7 +2609,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="31" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -2538,7 +2621,7 @@
         <v>104</v>
       </c>
       <c r="D31" s="1"/>
-      <c r="E31" s="1" t="s">
+      <c r="E31" s="18" t="s">
         <v>37</v>
       </c>
       <c r="F31" s="2" t="s">
@@ -2547,7 +2630,7 @@
       <c r="G31" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="H31">
+      <c r="H31" s="21">
         <f t="shared" si="1"/>
         <v>26</v>
       </c>
@@ -2569,7 +2652,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="32" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
         <f t="shared" si="0"/>
         <v>27</v>
@@ -2581,7 +2664,7 @@
         <v>104</v>
       </c>
       <c r="D32" s="1"/>
-      <c r="E32" s="1" t="s">
+      <c r="E32" s="18" t="s">
         <v>39</v>
       </c>
       <c r="F32" s="2" t="s">
@@ -2590,7 +2673,7 @@
       <c r="G32" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="H32">
+      <c r="H32" s="21">
         <f t="shared" si="1"/>
         <v>27</v>
       </c>
@@ -2612,7 +2695,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="33" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
         <f t="shared" si="0"/>
         <v>28</v>
@@ -2626,14 +2709,14 @@
       <c r="D33" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="E33" s="18" t="s">
         <v>73</v>
       </c>
       <c r="F33" s="2" t="s">
         <v>72</v>
       </c>
       <c r="G33" s="1"/>
-      <c r="H33">
+      <c r="H33" s="21">
         <f t="shared" si="1"/>
         <v>28</v>
       </c>
@@ -2653,7 +2736,7 @@
       </c>
       <c r="N33" s="1"/>
     </row>
-    <row r="34" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
         <f t="shared" si="0"/>
         <v>29</v>
@@ -2667,14 +2750,14 @@
       <c r="D34" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="E34" s="18" t="s">
         <v>75</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>74</v>
       </c>
       <c r="G34" s="1"/>
-      <c r="H34">
+      <c r="H34" s="21">
         <f t="shared" si="1"/>
         <v>29</v>
       </c>
@@ -2694,7 +2777,7 @@
       </c>
       <c r="N34" s="1"/>
     </row>
-    <row r="35" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
         <f t="shared" si="0"/>
         <v>30</v>
@@ -2706,7 +2789,7 @@
         <v>104</v>
       </c>
       <c r="D35" s="1"/>
-      <c r="E35" s="1" t="s">
+      <c r="E35" s="18" t="s">
         <v>49</v>
       </c>
       <c r="F35" s="2" t="s">
@@ -2715,7 +2798,7 @@
       <c r="G35" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="H35">
+      <c r="H35" s="21">
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
@@ -2733,7 +2816,7 @@
       </c>
       <c r="N35" s="1"/>
     </row>
-    <row r="36" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="5">
         <f t="shared" si="0"/>
         <v>31</v>
@@ -2745,7 +2828,7 @@
         <v>104</v>
       </c>
       <c r="D36" s="6"/>
-      <c r="E36" s="6" t="s">
+      <c r="E36" s="19" t="s">
         <v>51</v>
       </c>
       <c r="F36" s="5" t="s">
@@ -2754,7 +2837,7 @@
       <c r="G36" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="H36" s="8">
+      <c r="H36" s="22">
         <f t="shared" si="1"/>
         <v>31</v>
       </c>
@@ -2777,15 +2860,15 @@
       <c r="N36" s="6"/>
       <c r="O36" s="8"/>
     </row>
-    <row r="37" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2"/>
       <c r="B37" s="1"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="1"/>
-      <c r="E37" s="1"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="1"/>
-      <c r="H37">
+      <c r="C37" s="23"/>
+      <c r="D37" s="23"/>
+      <c r="E37" s="23"/>
+      <c r="F37" s="23"/>
+      <c r="G37" s="24"/>
+      <c r="H37" s="21">
         <f t="shared" si="1"/>
         <v>32</v>
       </c>
@@ -2797,18 +2880,18 @@
       <c r="M37" s="1"/>
       <c r="N37" s="1"/>
     </row>
-    <row r="38" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
         <f>A36+1</f>
         <v>32</v>
       </c>
       <c r="B38" s="1"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="1"/>
-      <c r="E38" s="1"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="1"/>
-      <c r="H38">
+      <c r="C38" s="25"/>
+      <c r="D38" s="25"/>
+      <c r="E38" s="25"/>
+      <c r="F38" s="25"/>
+      <c r="G38" s="26"/>
+      <c r="H38" s="21">
         <f t="shared" si="1"/>
         <v>33</v>
       </c>
@@ -2824,18 +2907,18 @@
       <c r="M38" s="1"/>
       <c r="N38" s="1"/>
     </row>
-    <row r="39" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="B39" s="1"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="1"/>
-      <c r="E39" s="1"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="1"/>
-      <c r="H39">
+      <c r="C39" s="25"/>
+      <c r="D39" s="25"/>
+      <c r="E39" s="25"/>
+      <c r="F39" s="25"/>
+      <c r="G39" s="26"/>
+      <c r="H39" s="21">
         <f t="shared" si="1"/>
         <v>34</v>
       </c>
@@ -2849,18 +2932,18 @@
       <c r="M39" s="1"/>
       <c r="N39" s="1"/>
     </row>
-    <row r="40" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
       <c r="B40" s="1"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="1"/>
-      <c r="E40" s="1"/>
-      <c r="F40" s="2"/>
-      <c r="G40" s="1"/>
-      <c r="H40">
+      <c r="C40" s="25"/>
+      <c r="D40" s="25"/>
+      <c r="E40" s="25"/>
+      <c r="F40" s="25"/>
+      <c r="G40" s="26"/>
+      <c r="H40" s="21">
         <f t="shared" si="1"/>
         <v>35</v>
       </c>
@@ -2874,18 +2957,18 @@
       <c r="M40" s="1"/>
       <c r="N40" s="1"/>
     </row>
-    <row r="41" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
       <c r="B41" s="1"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="1"/>
-      <c r="E41" s="1"/>
-      <c r="F41" s="2"/>
-      <c r="G41" s="1"/>
-      <c r="H41">
+      <c r="C41" s="25"/>
+      <c r="D41" s="25"/>
+      <c r="E41" s="25"/>
+      <c r="F41" s="25"/>
+      <c r="G41" s="26"/>
+      <c r="H41" s="21">
         <f t="shared" si="1"/>
         <v>36</v>
       </c>
@@ -2899,18 +2982,18 @@
       <c r="M41" s="1"/>
       <c r="N41" s="1"/>
     </row>
-    <row r="42" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
       <c r="B42" s="1"/>
-      <c r="C42" s="2"/>
-      <c r="D42" s="1"/>
-      <c r="E42" s="1"/>
-      <c r="F42" s="2"/>
-      <c r="G42" s="1"/>
-      <c r="H42">
+      <c r="C42" s="25"/>
+      <c r="D42" s="25"/>
+      <c r="E42" s="25"/>
+      <c r="F42" s="25"/>
+      <c r="G42" s="26"/>
+      <c r="H42" s="21">
         <f t="shared" si="1"/>
         <v>37</v>
       </c>
@@ -2926,18 +3009,18 @@
       <c r="M42" s="1"/>
       <c r="N42" s="1"/>
     </row>
-    <row r="43" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
       <c r="B43" s="1"/>
-      <c r="C43" s="2"/>
-      <c r="D43" s="1"/>
-      <c r="E43" s="1"/>
-      <c r="F43" s="2"/>
-      <c r="G43" s="1"/>
-      <c r="H43">
+      <c r="C43" s="25"/>
+      <c r="D43" s="25"/>
+      <c r="E43" s="25"/>
+      <c r="F43" s="25"/>
+      <c r="G43" s="26"/>
+      <c r="H43" s="21">
         <f t="shared" si="1"/>
         <v>38</v>
       </c>
@@ -2953,18 +3036,18 @@
       <c r="M43" s="1"/>
       <c r="N43" s="1"/>
     </row>
-    <row r="44" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
       <c r="B44" s="1"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="1"/>
-      <c r="E44" s="1"/>
-      <c r="F44" s="2"/>
-      <c r="G44" s="1"/>
-      <c r="H44">
+      <c r="C44" s="25"/>
+      <c r="D44" s="25"/>
+      <c r="E44" s="25"/>
+      <c r="F44" s="25"/>
+      <c r="G44" s="26"/>
+      <c r="H44" s="21">
         <f t="shared" si="1"/>
         <v>39</v>
       </c>
@@ -2978,18 +3061,18 @@
       <c r="M44" s="1"/>
       <c r="N44" s="1"/>
     </row>
-    <row r="45" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
       <c r="B45" s="1"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="1"/>
-      <c r="E45" s="1"/>
-      <c r="F45" s="2"/>
-      <c r="G45" s="1"/>
-      <c r="H45">
+      <c r="C45" s="25"/>
+      <c r="D45" s="25"/>
+      <c r="E45" s="25"/>
+      <c r="F45" s="25"/>
+      <c r="G45" s="26"/>
+      <c r="H45" s="21">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
@@ -3003,18 +3086,18 @@
       <c r="M45" s="1"/>
       <c r="N45" s="1"/>
     </row>
-    <row r="46" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
       <c r="B46" s="1"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="1"/>
-      <c r="E46" s="1"/>
-      <c r="F46" s="2"/>
-      <c r="G46" s="1"/>
-      <c r="H46">
+      <c r="C46" s="25"/>
+      <c r="D46" s="25"/>
+      <c r="E46" s="25"/>
+      <c r="F46" s="25"/>
+      <c r="G46" s="26"/>
+      <c r="H46" s="21">
         <f t="shared" si="1"/>
         <v>41</v>
       </c>
@@ -3028,18 +3111,18 @@
       <c r="M46" s="1"/>
       <c r="N46" s="1"/>
     </row>
-    <row r="47" spans="1:15" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:15" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
       <c r="B47" s="1"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="1"/>
-      <c r="E47" s="1"/>
-      <c r="F47" s="2"/>
-      <c r="G47" s="1"/>
-      <c r="H47">
+      <c r="C47" s="25"/>
+      <c r="D47" s="25"/>
+      <c r="E47" s="25"/>
+      <c r="F47" s="25"/>
+      <c r="G47" s="26"/>
+      <c r="H47" s="21">
         <f t="shared" si="1"/>
         <v>42</v>
       </c>
@@ -3063,7 +3146,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="C5:C8 F7:F8 J9:J13 C33:C34 C16 J38 J35:J36 J42:J43 C12 C18:C24" numberStoredAsText="1"/>
+    <ignoredError sqref="C5:C8 F7:F8 J9:J13 C33:C34 J38 J35:J36 J42:J43 C19:C24" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>